<commit_message>
Remove local choice row carriers and refine XLSX input handling
Store individual choice sources at issued field paths. Share XLSX decoding between template import and form reading, preserve authored names, read cached formula results, and correct engineering precision and blank list values.

Known follow-ups: decoding two distinct escaped sheet names can cause a false name collision; previous local choices/1 forms are rejected by the choices/2 reader. This commit preserves the current work for further revision.

Validation: check:release with 344 tests; independent consumer checks with 149 tests; native Excel save and local HTTP form import.
</commit_message>
<xml_diff>
--- a/test/fixtures/form-values-excel.xlsx
+++ b/test/fixtures/form-values-excel.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69F4D88B-6BB6-4F40-A1B9-1C85BCE9DE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E8921EF-E7BB-4E3C-8957-C9C684676D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14,9 +14,8 @@
     <sheet name="_sheetbind_lists" sheetId="4" state="veryHidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_sb_local_1">_sheetbind_lists!$A$1:$A$2</definedName>
-    <definedName name="_sb_local_2">_sheetbind_lists!$B$1</definedName>
-    <definedName name="_sb_object_sources">_sheetbind_lists!$C$1:$C$3</definedName>
+    <definedName name="_sb_list_1">_sheetbind_lists!$A$1:$A$2</definedName>
+    <definedName name="_sb_object_sources">_sheetbind_lists!$B$1:$B$3</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>Field</t>
   </si>
@@ -81,19 +80,16 @@
     <t>Good</t>
   </si>
   <si>
-    <t>_sb_local_1</t>
-  </si>
-  <si>
-    <t>sheetbind.choices/1</t>
+    <t>sheetbind.choices/2</t>
   </si>
   <si>
     <t>xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
   </si>
   <si>
-    <t>{"context":{},"dictionaries":{},"local":{"cell-30":{"sheet":"Choice","column":258,"values":[[{"id":"a","label":"Good"},{"id":"b","label":"xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
-  </si>
-  <si>
-    <t>xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx"}]]}}}</t>
+    <t>{"context":{},"dictionaries":{},"local":{"cell-30":{"$data.selected":[{"id":"a","label":"Good"},{"id":"b","label":"xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
+  </si>
+  <si>
+    <t>xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx"}]}}}</t>
   </si>
   <si>
     <t>006</t>
@@ -550,7 +546,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:257" x14ac:dyDescent="0.3">
@@ -558,7 +554,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:257" x14ac:dyDescent="0.3">
@@ -663,22 +659,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:IX2"/>
+  <dimension ref="A1:IW2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="257" max="257" width="2" hidden="1" customWidth="1"/>
-    <col min="258" max="258" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:258" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:257" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="IX1" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:258" hidden="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:257" hidden="1" x14ac:dyDescent="0.3">
       <c r="IW2" s="10" t="s">
         <v>13</v>
       </c>
@@ -686,7 +678,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Choose a listed value" error="Select a value from the dropdown list." sqref="A1" xr:uid="{00000000-0002-0000-0200-000000000000}">
-      <formula1>INDIRECT(IF(INDEX(_sb_local_2,$IX1)="#input",ADDRESS(ROW(),COLUMN()),INDEX(_sb_local_2,$IX1)))</formula1>
+      <formula1>_sb_list_1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -696,31 +688,28 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="11" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="B2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="11" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="11" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C3" s="11" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>